<commit_message>
further refined core variables data dict to reflect only essential core vars
</commit_message>
<xml_diff>
--- a/Get variables/core_var_data_dict.xlsx
+++ b/Get variables/core_var_data_dict.xlsx
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="145">
   <si>
     <t>General health  </t>
   </si>
@@ -156,15 +156,9 @@
     <t>Seen doctor (GP) for nerves, anxiety, tension or depression</t>
   </si>
   <si>
-    <t>Place of birth in UK - east co-ordinate</t>
-  </si>
-  <si>
     <t>Early life factors  </t>
   </si>
   <si>
-    <t>Place of birth in UK - north co-ordinate</t>
-  </si>
-  <si>
     <t>Home area population density - urban or rural</t>
   </si>
   <si>
@@ -219,9 +213,6 @@
     <t>Maternal smoking around birth</t>
   </si>
   <si>
-    <t>Early life factors </t>
-  </si>
-  <si>
     <t>Alcohol consumed</t>
   </si>
   <si>
@@ -297,12 +288,6 @@
     <t>yes</t>
   </si>
   <si>
-    <t>place_birth_east</t>
-  </si>
-  <si>
-    <t>place_birth_north</t>
-  </si>
-  <si>
     <t>adopted</t>
   </si>
   <si>
@@ -405,9 +390,6 @@
     <t>day_sleepiness</t>
   </si>
   <si>
-    <t>alcohol</t>
-  </si>
-  <si>
     <t>Index of Multiple Deprivation (England)</t>
   </si>
   <si>
@@ -493,6 +475,9 @@
   </si>
   <si>
     <t>BMR</t>
+  </si>
+  <si>
+    <t>alcohol_yesterday</t>
   </si>
 </sst>
 </file>
@@ -906,22 +891,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="B1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
       <c r="E1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -935,13 +920,13 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -955,13 +940,13 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -975,13 +960,13 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -995,13 +980,13 @@
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1015,13 +1000,13 @@
         <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1061,22 +1046,22 @@
   <sheetData>
     <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>75</v>
-      </c>
       <c r="E1" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1090,13 +1075,13 @@
         <v>9</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1110,13 +1095,13 @@
         <v>9</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1134,7 +1119,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="55.42578125" customWidth="1"/>
@@ -1143,164 +1128,118 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="B1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
       <c r="E1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>130</v>
+        <v>20118</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>129</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>38</v>
+      <c r="A3" s="3">
+        <v>26410</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>118</v>
       </c>
       <c r="D3" t="s">
-        <v>85</v>
+        <v>119</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>20118</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>9</v>
+      <c r="A4" s="3">
+        <v>26427</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>118</v>
       </c>
       <c r="D4" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
-        <v>26410</v>
+        <v>26426</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" t="s">
         <v>121</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D5" t="s">
-        <v>125</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
-        <v>26427</v>
-      </c>
-      <c r="B6" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D6" t="s">
-        <v>126</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F6" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>26426</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" t="s">
-        <v>127</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F7" t="s">
-        <v>128</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=130"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=130"/>
-    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072"/>
-    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=129"/>
-    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=129"/>
-    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072"/>
-    <hyperlink ref="A4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20118"/>
-    <hyperlink ref="B4" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20118"/>
-    <hyperlink ref="C4" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024"/>
-    <hyperlink ref="A5" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26410"/>
-    <hyperlink ref="B5" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26410"/>
-    <hyperlink ref="A6" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26427"/>
-    <hyperlink ref="B6" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26427"/>
-    <hyperlink ref="A7" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26426"/>
-    <hyperlink ref="B7" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26426"/>
-    <hyperlink ref="C5" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701"/>
-    <hyperlink ref="C6" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701"/>
-    <hyperlink ref="C7" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20118"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20118"/>
+    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024"/>
+    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26410"/>
+    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26410"/>
+    <hyperlink ref="A4" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26427"/>
+    <hyperlink ref="B4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26427"/>
+    <hyperlink ref="A5" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26426"/>
+    <hyperlink ref="B5" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26426"/>
+    <hyperlink ref="C3" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701"/>
+    <hyperlink ref="C4" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701"/>
+    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1312,27 +1251,27 @@
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="48.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="B1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
       <c r="E1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1340,19 +1279,19 @@
         <v>845</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1360,19 +1299,19 @@
         <v>6138</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1380,19 +1319,19 @@
         <v>6142</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1400,19 +1339,19 @@
         <v>20119</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1420,19 +1359,19 @@
         <v>3426</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1440,19 +1379,19 @@
         <v>826</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1460,19 +1399,19 @@
         <v>132</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1505,7 +1444,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="35.7109375" bestFit="1" customWidth="1"/>
@@ -1515,22 +1454,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="B1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
       <c r="E1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1538,19 +1477,19 @@
         <v>1767</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1558,19 +1497,19 @@
         <v>20022</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1578,19 +1517,19 @@
         <v>120</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1598,19 +1537,19 @@
         <v>1677</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1618,19 +1557,19 @@
         <v>20115</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1638,19 +1577,19 @@
         <v>1647</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1658,19 +1597,19 @@
         <v>1707</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1678,59 +1617,19 @@
         <v>1787</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>130</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" t="s">
-        <v>84</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F10" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>129</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" t="s">
-        <v>85</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1759,12 +1658,6 @@
     <hyperlink ref="A9" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1787"/>
     <hyperlink ref="B9" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1787"/>
     <hyperlink ref="C9" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033"/>
-    <hyperlink ref="A10" r:id="rId25" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=130"/>
-    <hyperlink ref="B10" r:id="rId26" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=130"/>
-    <hyperlink ref="C10" r:id="rId27" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072"/>
-    <hyperlink ref="A11" r:id="rId28" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=129"/>
-    <hyperlink ref="B11" r:id="rId29" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=129"/>
-    <hyperlink ref="C11" r:id="rId30" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1785,22 +1678,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
       <c r="E1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1808,19 +1701,19 @@
         <v>20116</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1828,19 +1721,19 @@
         <v>1558</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1854,13 +1747,13 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1874,13 +1767,13 @@
         <v>4</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1894,13 +1787,13 @@
         <v>4</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1908,19 +1801,19 @@
         <v>6146</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1934,13 +1827,13 @@
         <v>0</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1954,13 +1847,13 @@
         <v>34</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1974,13 +1867,13 @@
         <v>34</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -2029,22 +1922,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>75</v>
-      </c>
       <c r="E1" s="11" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -2052,19 +1945,19 @@
         <v>1050</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2072,19 +1965,19 @@
         <v>1060</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2139,26 +2032,27 @@
   <cols>
     <col min="1" max="1" width="14.85546875" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="B1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
       <c r="E1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2166,16 +2060,16 @@
         <v>1160</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2183,16 +2077,16 @@
         <v>1170</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2200,16 +2094,16 @@
         <v>1180</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2217,16 +2111,16 @@
         <v>1190</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2234,16 +2128,16 @@
         <v>1200</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2251,16 +2145,16 @@
         <v>1210</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2268,16 +2162,16 @@
         <v>1220</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D8" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2285,19 +2179,19 @@
         <v>100580</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D9" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -2335,22 +2229,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="B1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" t="s">
-        <v>75</v>
-      </c>
       <c r="E1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2364,13 +2258,13 @@
         <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2384,13 +2278,13 @@
         <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2404,13 +2298,13 @@
         <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2424,13 +2318,13 @@
         <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2444,13 +2338,13 @@
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2464,13 +2358,13 @@
         <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2484,13 +2378,13 @@
         <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2504,13 +2398,13 @@
         <v>28</v>
       </c>
       <c r="D9" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2524,13 +2418,13 @@
         <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2544,13 +2438,13 @@
         <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2564,13 +2458,13 @@
         <v>31</v>
       </c>
       <c r="D12" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2584,13 +2478,13 @@
         <v>31</v>
       </c>
       <c r="D13" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F13" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -2637,6 +2531,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002D5D40E36B58B0418A5C0DC6F6A2845B" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a816bc34d4292327d4a371c81c74c3a5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xmlns:ns4="301edac2-2a5a-4564-9129-5d780cc3d1d3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="773e6490813a0ac7eb54afe68e0456d4" ns3:_="" ns4:_="">
     <xsd:import namespace="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
@@ -2851,15 +2754,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2869,6 +2763,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD47ECBE-2CA4-4905-9B25-5B5DD8B09919}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2887,18 +2789,9 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -2906,6 +2799,7 @@
     <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>

</xml_diff>

<commit_message>
removed job_code and BMR which are variables not included in core dataset basket
</commit_message>
<xml_diff>
--- a/Get variables/core_var_data_dict.xlsx
+++ b/Get variables/core_var_data_dict.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arogusk2\OneDrive - University of Edinburgh\HELIOS-BD\Side Projects\BioBank Project\Git\biobank-time-dimensions\Get variables\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC6A7EA-CE6C-4CD1-9431-ED3B2EC0FD9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" tabRatio="849" activeTab="8"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="849" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Primary demographics" sheetId="2" r:id="rId1"/>
@@ -27,23 +28,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="141">
   <si>
     <t>General health  </t>
   </si>
@@ -114,9 +104,6 @@
     <t>Body composition by impedance  </t>
   </si>
   <si>
-    <t>Basal metabolic rate</t>
-  </si>
-  <si>
     <t>Body fat percentage</t>
   </si>
   <si>
@@ -180,9 +167,6 @@
     <t>Current employment status - corrected</t>
   </si>
   <si>
-    <t>Job code at visit - entered</t>
-  </si>
-  <si>
     <t>Job involves night shift work</t>
   </si>
   <si>
@@ -417,9 +401,6 @@
     <t>employed_corrected</t>
   </si>
   <si>
-    <t>job</t>
-  </si>
-  <si>
     <t>Attendance/disability/mobility allowance</t>
   </si>
   <si>
@@ -472,9 +453,6 @@
   </si>
   <si>
     <t>disability_self_report</t>
-  </si>
-  <si>
-    <t>BMR</t>
   </si>
   <si>
     <t>alcohol_yesterday</t>
@@ -483,8 +461,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -504,13 +482,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -537,7 +508,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -552,9 +523,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
@@ -880,7 +848,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -891,22 +859,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -920,13 +888,13 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -940,13 +908,13 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -960,13 +928,13 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -980,13 +948,13 @@
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1000,32 +968,32 @@
         <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=31"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=31"/>
-    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100094"/>
-    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21003"/>
-    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21003"/>
-    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024"/>
-    <hyperlink ref="A4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=34"/>
-    <hyperlink ref="B4" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=34"/>
-    <hyperlink ref="C4" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100094"/>
-    <hyperlink ref="A5" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=52"/>
-    <hyperlink ref="B5" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=52"/>
-    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100094"/>
-    <hyperlink ref="A6" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21000"/>
-    <hyperlink ref="B6" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21000"/>
-    <hyperlink ref="C6" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100065"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=31" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=31" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100094" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21003" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21003" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="A4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=34" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="B4" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=34" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="C4" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100094" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="A5" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=52" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="B5" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=52" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100094" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="A6" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21000" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B6" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21000" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="C6" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100065" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId16"/>
@@ -1033,7 +1001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1046,22 +1014,22 @@
   <sheetData>
     <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1075,13 +1043,13 @@
         <v>9</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1095,30 +1063,30 @@
         <v>9</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=54"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=54"/>
-    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024"/>
-    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=53"/>
-    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=53"/>
-    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=54" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=54" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=53" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=53" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1128,22 +1096,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1151,19 +1119,19 @@
         <v>20118</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1171,19 +1139,19 @@
         <v>26410</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1191,19 +1159,19 @@
         <v>26427</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" t="s">
         <v>118</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" t="s">
         <v>120</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F4" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1211,43 +1179,43 @@
         <v>26426</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20118"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20118"/>
-    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024"/>
-    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26410"/>
-    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26410"/>
-    <hyperlink ref="A4" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26427"/>
-    <hyperlink ref="B4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26427"/>
-    <hyperlink ref="A5" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26426"/>
-    <hyperlink ref="B5" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26426"/>
-    <hyperlink ref="C3" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701"/>
-    <hyperlink ref="C4" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701"/>
-    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20118" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20118" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100024" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
+    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26410" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
+    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26410" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="A4" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26427" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="B4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26427" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="A5" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26426" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
+    <hyperlink ref="B5" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=26426" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
+    <hyperlink ref="C3" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
+    <hyperlink ref="C4" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
+    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=701" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="48.140625" bestFit="1" customWidth="1"/>
@@ -1256,22 +1224,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1279,19 +1247,19 @@
         <v>845</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="D2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1299,19 +1267,19 @@
         <v>6138</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1319,19 +1287,19 @@
         <v>6142</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1339,19 +1307,19 @@
         <v>20119</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1359,19 +1327,19 @@
         <v>3426</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1379,71 +1347,48 @@
         <v>826</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>132</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=845"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=845"/>
-    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100063"/>
-    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=6138"/>
-    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=6138"/>
-    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100063"/>
-    <hyperlink ref="A4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=6142"/>
-    <hyperlink ref="B4" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=6142"/>
-    <hyperlink ref="C4" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100064"/>
-    <hyperlink ref="A5" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20119"/>
-    <hyperlink ref="B5" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20119"/>
-    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100064"/>
-    <hyperlink ref="A8" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=132"/>
-    <hyperlink ref="B8" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=132"/>
-    <hyperlink ref="C8" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100073"/>
-    <hyperlink ref="A6" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3426"/>
-    <hyperlink ref="B6" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3426"/>
-    <hyperlink ref="C6" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100064"/>
-    <hyperlink ref="A7" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=826"/>
-    <hyperlink ref="B7" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=826"/>
-    <hyperlink ref="C7" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100064"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=845" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=845" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100063" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
+    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=6138" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
+    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=6138" xr:uid="{00000000-0004-0000-0300-000004000000}"/>
+    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100063" xr:uid="{00000000-0004-0000-0300-000005000000}"/>
+    <hyperlink ref="A4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=6142" xr:uid="{00000000-0004-0000-0300-000006000000}"/>
+    <hyperlink ref="B4" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=6142" xr:uid="{00000000-0004-0000-0300-000007000000}"/>
+    <hyperlink ref="C4" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100064" xr:uid="{00000000-0004-0000-0300-000008000000}"/>
+    <hyperlink ref="A5" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20119" xr:uid="{00000000-0004-0000-0300-000009000000}"/>
+    <hyperlink ref="B5" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20119" xr:uid="{00000000-0004-0000-0300-00000A000000}"/>
+    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100064" xr:uid="{00000000-0004-0000-0300-00000B000000}"/>
+    <hyperlink ref="A6" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3426" xr:uid="{00000000-0004-0000-0300-00000F000000}"/>
+    <hyperlink ref="B6" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3426" xr:uid="{00000000-0004-0000-0300-000010000000}"/>
+    <hyperlink ref="C6" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100064" xr:uid="{00000000-0004-0000-0300-000011000000}"/>
+    <hyperlink ref="A7" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=826" xr:uid="{00000000-0004-0000-0300-000012000000}"/>
+    <hyperlink ref="B7" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=826" xr:uid="{00000000-0004-0000-0300-000013000000}"/>
+    <hyperlink ref="C7" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100064" xr:uid="{00000000-0004-0000-0300-000014000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1454,22 +1399,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1477,19 +1422,19 @@
         <v>1767</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1497,19 +1442,19 @@
         <v>20022</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1517,19 +1462,19 @@
         <v>120</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1537,19 +1482,19 @@
         <v>1677</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1557,19 +1502,19 @@
         <v>20115</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1577,19 +1522,19 @@
         <v>1647</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1597,19 +1542,19 @@
         <v>1707</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1617,54 +1562,54 @@
         <v>1787</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1767"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1767"/>
-    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033"/>
-    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20022"/>
-    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20022"/>
-    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072"/>
-    <hyperlink ref="A4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=120"/>
-    <hyperlink ref="B4" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=120"/>
-    <hyperlink ref="C4" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072"/>
-    <hyperlink ref="A5" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1677"/>
-    <hyperlink ref="B5" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1677"/>
-    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033"/>
-    <hyperlink ref="A6" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20115"/>
-    <hyperlink ref="B6" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20115"/>
-    <hyperlink ref="C6" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072"/>
-    <hyperlink ref="A7" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1647"/>
-    <hyperlink ref="B7" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1647"/>
-    <hyperlink ref="C7" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033"/>
-    <hyperlink ref="A8" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1707"/>
-    <hyperlink ref="B8" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1707"/>
-    <hyperlink ref="C8" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033"/>
-    <hyperlink ref="A9" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1787"/>
-    <hyperlink ref="B9" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1787"/>
-    <hyperlink ref="C9" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1767" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1767" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
+    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
+    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20022" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
+    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20022" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
+    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
+    <hyperlink ref="A4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=120" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
+    <hyperlink ref="B4" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=120" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
+    <hyperlink ref="C4" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
+    <hyperlink ref="A5" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1677" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
+    <hyperlink ref="B5" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1677" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
+    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
+    <hyperlink ref="A6" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20115" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
+    <hyperlink ref="B6" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20115" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
+    <hyperlink ref="C6" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100072" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
+    <hyperlink ref="A7" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1647" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
+    <hyperlink ref="B7" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1647" xr:uid="{00000000-0004-0000-0400-000010000000}"/>
+    <hyperlink ref="C7" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033" xr:uid="{00000000-0004-0000-0400-000011000000}"/>
+    <hyperlink ref="A8" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1707" xr:uid="{00000000-0004-0000-0400-000012000000}"/>
+    <hyperlink ref="B8" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1707" xr:uid="{00000000-0004-0000-0400-000013000000}"/>
+    <hyperlink ref="C8" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033" xr:uid="{00000000-0004-0000-0400-000014000000}"/>
+    <hyperlink ref="A9" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1787" xr:uid="{00000000-0004-0000-0400-000015000000}"/>
+    <hyperlink ref="B9" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=1787" xr:uid="{00000000-0004-0000-0400-000016000000}"/>
+    <hyperlink ref="C9" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100033" xr:uid="{00000000-0004-0000-0400-000017000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1677,63 +1622,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="D1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>20116</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="11">
+        <v>1558</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D3" t="s">
         <v>130</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="12">
-        <v>1558</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" t="s">
-        <v>133</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1747,171 +1692,171 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
+      <c r="A5" s="13">
         <v>137</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="14">
+      <c r="A6" s="13">
         <v>20003</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="13" t="s">
         <v>4</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
+      <c r="A7" s="11">
         <v>6146</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>126</v>
+      <c r="B7" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>123</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="14">
+      <c r="A8" s="13">
         <v>2188</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="13" t="s">
         <v>0</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="14">
+      <c r="A9" s="13">
         <v>2100</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="13">
+        <v>2090</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="E9" s="6" t="s">
+      <c r="C10" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="14">
-        <v>2090</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>91</v>
-      </c>
       <c r="E10" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=20116"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=20116"/>
-    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100058"/>
-    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1558"/>
-    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1558"/>
-    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100051"/>
-    <hyperlink ref="A5" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=137"/>
-    <hyperlink ref="B5" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=137"/>
-    <hyperlink ref="C5" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100075"/>
-    <hyperlink ref="A6" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20003"/>
-    <hyperlink ref="B6" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20003"/>
-    <hyperlink ref="C6" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100075"/>
-    <hyperlink ref="A4" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2178"/>
-    <hyperlink ref="B4" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2178"/>
-    <hyperlink ref="C4" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100042"/>
-    <hyperlink ref="A7" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=6146"/>
-    <hyperlink ref="B7" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=6146"/>
-    <hyperlink ref="C7" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100067"/>
-    <hyperlink ref="A8" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2188"/>
-    <hyperlink ref="B8" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2188"/>
-    <hyperlink ref="C8" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100042"/>
-    <hyperlink ref="A9" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2100"/>
-    <hyperlink ref="B9" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2100"/>
-    <hyperlink ref="C9" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100060"/>
-    <hyperlink ref="A10" r:id="rId25" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2090"/>
-    <hyperlink ref="B10" r:id="rId26" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2090"/>
-    <hyperlink ref="C10" r:id="rId27" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100060"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=20116" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=20116" xr:uid="{00000000-0004-0000-0500-000001000000}"/>
+    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100058" xr:uid="{00000000-0004-0000-0500-000002000000}"/>
+    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1558" xr:uid="{00000000-0004-0000-0500-000003000000}"/>
+    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1558" xr:uid="{00000000-0004-0000-0500-000004000000}"/>
+    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100051" xr:uid="{00000000-0004-0000-0500-000005000000}"/>
+    <hyperlink ref="A5" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=137" xr:uid="{00000000-0004-0000-0500-000006000000}"/>
+    <hyperlink ref="B5" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=137" xr:uid="{00000000-0004-0000-0500-000007000000}"/>
+    <hyperlink ref="C5" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100075" xr:uid="{00000000-0004-0000-0500-000008000000}"/>
+    <hyperlink ref="A6" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20003" xr:uid="{00000000-0004-0000-0500-000009000000}"/>
+    <hyperlink ref="B6" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20003" xr:uid="{00000000-0004-0000-0500-00000A000000}"/>
+    <hyperlink ref="C6" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100075" xr:uid="{00000000-0004-0000-0500-00000B000000}"/>
+    <hyperlink ref="A4" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2178" xr:uid="{00000000-0004-0000-0500-00000C000000}"/>
+    <hyperlink ref="B4" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2178" xr:uid="{00000000-0004-0000-0500-00000D000000}"/>
+    <hyperlink ref="C4" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100042" xr:uid="{00000000-0004-0000-0500-00000E000000}"/>
+    <hyperlink ref="A7" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=6146" xr:uid="{00000000-0004-0000-0500-00000F000000}"/>
+    <hyperlink ref="B7" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=6146" xr:uid="{00000000-0004-0000-0500-000010000000}"/>
+    <hyperlink ref="C7" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100067" xr:uid="{00000000-0004-0000-0500-000011000000}"/>
+    <hyperlink ref="A8" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2188" xr:uid="{00000000-0004-0000-0500-000012000000}"/>
+    <hyperlink ref="B8" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2188" xr:uid="{00000000-0004-0000-0500-000013000000}"/>
+    <hyperlink ref="C8" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100042" xr:uid="{00000000-0004-0000-0500-000014000000}"/>
+    <hyperlink ref="A9" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2100" xr:uid="{00000000-0004-0000-0500-000015000000}"/>
+    <hyperlink ref="B9" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2100" xr:uid="{00000000-0004-0000-0500-000016000000}"/>
+    <hyperlink ref="C9" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100060" xr:uid="{00000000-0004-0000-0500-000017000000}"/>
+    <hyperlink ref="A10" r:id="rId25" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2090" xr:uid="{00000000-0004-0000-0500-000018000000}"/>
+    <hyperlink ref="B10" r:id="rId26" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2090" xr:uid="{00000000-0004-0000-0500-000019000000}"/>
+    <hyperlink ref="C10" r:id="rId27" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100060" xr:uid="{00000000-0004-0000-0500-00001A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1921,112 +1866,112 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="F1" s="11" t="s">
-        <v>76</v>
+      <c r="E1" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="12">
+      <c r="A2" s="11">
         <v>1050</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>122</v>
+      <c r="E2" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="12">
+      <c r="A3" s="11">
         <v>1060</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>122</v>
+      <c r="E3" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1050"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1050"/>
-    <hyperlink ref="A3" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1060"/>
-    <hyperlink ref="B3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1060"/>
-    <hyperlink ref="C2" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100055"/>
-    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100055"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1050" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1050" xr:uid="{00000000-0004-0000-0600-000001000000}"/>
+    <hyperlink ref="A3" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1060" xr:uid="{00000000-0004-0000-0600-000002000000}"/>
+    <hyperlink ref="B3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=1060" xr:uid="{00000000-0004-0000-0600-000003000000}"/>
+    <hyperlink ref="C2" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100055" xr:uid="{00000000-0004-0000-0600-000004000000}"/>
+    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?tk=mx0s1o0mwTsDkrHR2d3hWdDShzSaCC1O349411&amp;id=100055" xr:uid="{00000000-0004-0000-0600-000005000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2037,22 +1982,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2060,16 +2005,16 @@
         <v>1160</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2077,16 +2022,16 @@
         <v>1170</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2094,16 +2039,16 @@
         <v>1180</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2111,16 +2056,16 @@
         <v>1190</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2128,16 +2073,16 @@
         <v>1200</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2145,16 +2090,16 @@
         <v>1210</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2162,16 +2107,16 @@
         <v>1220</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2179,40 +2124,40 @@
         <v>100580</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1160"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1160"/>
-    <hyperlink ref="A3" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1170"/>
-    <hyperlink ref="B3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1170"/>
-    <hyperlink ref="A4" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1180"/>
-    <hyperlink ref="B4" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1180"/>
-    <hyperlink ref="A5" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1190"/>
-    <hyperlink ref="B5" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1190"/>
-    <hyperlink ref="A6" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1200"/>
-    <hyperlink ref="B6" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1200"/>
-    <hyperlink ref="A7" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1210"/>
-    <hyperlink ref="B7" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1210"/>
-    <hyperlink ref="A8" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1220"/>
-    <hyperlink ref="B8" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1220"/>
-    <hyperlink ref="A9" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=100580"/>
-    <hyperlink ref="B9" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=100580"/>
-    <hyperlink ref="C9" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100100"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1160" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1160" xr:uid="{00000000-0004-0000-0700-000001000000}"/>
+    <hyperlink ref="A3" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1170" xr:uid="{00000000-0004-0000-0700-000002000000}"/>
+    <hyperlink ref="B3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1170" xr:uid="{00000000-0004-0000-0700-000003000000}"/>
+    <hyperlink ref="A4" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1180" xr:uid="{00000000-0004-0000-0700-000004000000}"/>
+    <hyperlink ref="B4" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1180" xr:uid="{00000000-0004-0000-0700-000005000000}"/>
+    <hyperlink ref="A5" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1190" xr:uid="{00000000-0004-0000-0700-000006000000}"/>
+    <hyperlink ref="B5" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1190" xr:uid="{00000000-0004-0000-0700-000007000000}"/>
+    <hyperlink ref="A6" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1200" xr:uid="{00000000-0004-0000-0700-000008000000}"/>
+    <hyperlink ref="B6" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1200" xr:uid="{00000000-0004-0000-0700-000009000000}"/>
+    <hyperlink ref="A7" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1210" xr:uid="{00000000-0004-0000-0700-00000A000000}"/>
+    <hyperlink ref="B7" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1210" xr:uid="{00000000-0004-0000-0700-00000B000000}"/>
+    <hyperlink ref="A8" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1220" xr:uid="{00000000-0004-0000-0700-00000C000000}"/>
+    <hyperlink ref="B8" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1220" xr:uid="{00000000-0004-0000-0700-00000D000000}"/>
+    <hyperlink ref="A9" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=100580" xr:uid="{00000000-0004-0000-0700-00000E000000}"/>
+    <hyperlink ref="B9" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=100580" xr:uid="{00000000-0004-0000-0700-00000F000000}"/>
+    <hyperlink ref="C9" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100100" xr:uid="{00000000-0004-0000-0700-000010000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId18"/>
@@ -2220,8 +2165,8 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="57.5703125" bestFit="1" customWidth="1"/>
@@ -2229,22 +2174,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2258,13 +2203,13 @@
         <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2278,13 +2223,13 @@
         <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2298,13 +2243,13 @@
         <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2318,18 +2263,18 @@
         <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>23105</v>
+        <v>23099</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>23</v>
@@ -2338,205 +2283,181 @@
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>143</v>
+        <v>99</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>23099</v>
+        <v>21001</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>21001</v>
+        <v>46</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>47</v>
+        <v>3063</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F10" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>3063</v>
+        <v>3062</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="D11" t="s">
         <v>105</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F11" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>3062</v>
+        <v>3064</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F12" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>3064</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" t="s">
-        <v>106</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=90012"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=90012"/>
-    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=1009"/>
-    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=4079"/>
-    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=4079"/>
-    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100011"/>
-    <hyperlink ref="A4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=102"/>
-    <hyperlink ref="B4" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=102"/>
-    <hyperlink ref="C4" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100011"/>
-    <hyperlink ref="A5" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=4080"/>
-    <hyperlink ref="B5" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=4080"/>
-    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100011"/>
-    <hyperlink ref="A6" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=23105"/>
-    <hyperlink ref="B6" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=23105"/>
-    <hyperlink ref="C6" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100009"/>
-    <hyperlink ref="A7" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=23099"/>
-    <hyperlink ref="B7" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=23099"/>
-    <hyperlink ref="C7" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100009"/>
-    <hyperlink ref="A8" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21001"/>
-    <hyperlink ref="B8" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21001"/>
-    <hyperlink ref="C8" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100010"/>
-    <hyperlink ref="A9" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=46"/>
-    <hyperlink ref="B9" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=46"/>
-    <hyperlink ref="C9" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100019"/>
-    <hyperlink ref="A10" r:id="rId25" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=47"/>
-    <hyperlink ref="B10" r:id="rId26" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=47"/>
-    <hyperlink ref="C10" r:id="rId27" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100019"/>
-    <hyperlink ref="A11" r:id="rId28" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3063"/>
-    <hyperlink ref="B11" r:id="rId29" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3063"/>
-    <hyperlink ref="C11" r:id="rId30" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100020"/>
-    <hyperlink ref="A12" r:id="rId31" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3062"/>
-    <hyperlink ref="B12" r:id="rId32" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3062"/>
-    <hyperlink ref="C12" r:id="rId33" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100020"/>
-    <hyperlink ref="A13" r:id="rId34" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3064"/>
-    <hyperlink ref="B13" r:id="rId35" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3064"/>
-    <hyperlink ref="C13" r:id="rId36" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100020"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=90012" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=90012" xr:uid="{00000000-0004-0000-0800-000001000000}"/>
+    <hyperlink ref="C2" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=1009" xr:uid="{00000000-0004-0000-0800-000002000000}"/>
+    <hyperlink ref="A3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=4079" xr:uid="{00000000-0004-0000-0800-000003000000}"/>
+    <hyperlink ref="B3" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=4079" xr:uid="{00000000-0004-0000-0800-000004000000}"/>
+    <hyperlink ref="C3" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100011" xr:uid="{00000000-0004-0000-0800-000005000000}"/>
+    <hyperlink ref="A4" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=102" xr:uid="{00000000-0004-0000-0800-000006000000}"/>
+    <hyperlink ref="B4" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=102" xr:uid="{00000000-0004-0000-0800-000007000000}"/>
+    <hyperlink ref="C4" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100011" xr:uid="{00000000-0004-0000-0800-000008000000}"/>
+    <hyperlink ref="A5" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=4080" xr:uid="{00000000-0004-0000-0800-000009000000}"/>
+    <hyperlink ref="B5" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=4080" xr:uid="{00000000-0004-0000-0800-00000A000000}"/>
+    <hyperlink ref="C5" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100011" xr:uid="{00000000-0004-0000-0800-00000B000000}"/>
+    <hyperlink ref="A6" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=23099" xr:uid="{00000000-0004-0000-0800-00000F000000}"/>
+    <hyperlink ref="B6" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=23099" xr:uid="{00000000-0004-0000-0800-000010000000}"/>
+    <hyperlink ref="C6" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100009" xr:uid="{00000000-0004-0000-0800-000011000000}"/>
+    <hyperlink ref="A7" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21001" xr:uid="{00000000-0004-0000-0800-000012000000}"/>
+    <hyperlink ref="B7" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=21001" xr:uid="{00000000-0004-0000-0800-000013000000}"/>
+    <hyperlink ref="C7" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100010" xr:uid="{00000000-0004-0000-0800-000014000000}"/>
+    <hyperlink ref="A8" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=46" xr:uid="{00000000-0004-0000-0800-000015000000}"/>
+    <hyperlink ref="B8" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=46" xr:uid="{00000000-0004-0000-0800-000016000000}"/>
+    <hyperlink ref="C8" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100019" xr:uid="{00000000-0004-0000-0800-000017000000}"/>
+    <hyperlink ref="A9" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=47" xr:uid="{00000000-0004-0000-0800-000018000000}"/>
+    <hyperlink ref="B9" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=47" xr:uid="{00000000-0004-0000-0800-000019000000}"/>
+    <hyperlink ref="C9" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100019" xr:uid="{00000000-0004-0000-0800-00001A000000}"/>
+    <hyperlink ref="A10" r:id="rId25" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3063" xr:uid="{00000000-0004-0000-0800-00001B000000}"/>
+    <hyperlink ref="B10" r:id="rId26" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3063" xr:uid="{00000000-0004-0000-0800-00001C000000}"/>
+    <hyperlink ref="C10" r:id="rId27" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100020" xr:uid="{00000000-0004-0000-0800-00001D000000}"/>
+    <hyperlink ref="A11" r:id="rId28" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3062" xr:uid="{00000000-0004-0000-0800-00001E000000}"/>
+    <hyperlink ref="B11" r:id="rId29" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3062" xr:uid="{00000000-0004-0000-0800-00001F000000}"/>
+    <hyperlink ref="C11" r:id="rId30" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100020" xr:uid="{00000000-0004-0000-0800-000020000000}"/>
+    <hyperlink ref="A12" r:id="rId31" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3064" xr:uid="{00000000-0004-0000-0800-000021000000}"/>
+    <hyperlink ref="B12" r:id="rId32" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=3064" xr:uid="{00000000-0004-0000-0800-000022000000}"/>
+    <hyperlink ref="C12" r:id="rId33" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100020" xr:uid="{00000000-0004-0000-0800-000023000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2755,17 +2676,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2790,18 +2721,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
amending cor var data dict to reflect 'data collection timing' vars
</commit_message>
<xml_diff>
--- a/Get variables/core_var_data_dict.xlsx
+++ b/Get variables/core_var_data_dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arogusk2\OneDrive - University of Edinburgh\HELIOS-BD\Side Projects\BioBank Project\Git\biobank-time-dimensions\Get variables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC6A7EA-CE6C-4CD1-9431-ED3B2EC0FD9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B437E2A0-61B2-44D4-AF16-8B33579B967B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="849" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1875" windowWidth="29040" windowHeight="15840" tabRatio="849" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Primary demographics" sheetId="2" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="Seasonal" sheetId="13" r:id="rId7"/>
     <sheet name="Sleep" sheetId="10" r:id="rId8"/>
     <sheet name="Physical measure summary" sheetId="3" r:id="rId9"/>
+    <sheet name="Data Collection Timings" sheetId="14" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="175">
   <si>
     <t>General health  </t>
   </si>
@@ -456,6 +457,108 @@
   </si>
   <si>
     <t>alcohol_yesterday</t>
+  </si>
+  <si>
+    <t>Biometrics duration</t>
+  </si>
+  <si>
+    <t>Conclusion duration</t>
+  </si>
+  <si>
+    <t>ECG during exercise duration</t>
+  </si>
+  <si>
+    <t>Eye measures duration</t>
+  </si>
+  <si>
+    <t>Sample collection duration</t>
+  </si>
+  <si>
+    <t>Touchscreen duration</t>
+  </si>
+  <si>
+    <t>Verbal interview duration</t>
+  </si>
+  <si>
+    <t>Biometrics sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Brain MRI sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Cardiac monitor sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Carotid ultrasound sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Chest MRI sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Conclusion sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Consent sign-off timestamp</t>
+  </si>
+  <si>
+    <t>DXA assessment sign-off timestamp</t>
+  </si>
+  <si>
+    <t>ECG at rest sign-off timestamp</t>
+  </si>
+  <si>
+    <t>ECG during exercise sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Eye measures sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Imaging screening sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Measurement/Impedance sign-off timestamp (pilot)</t>
+  </si>
+  <si>
+    <t>Pilot Spirometry sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Reception sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Sample collection sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Touchscreen cognitive sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Touchscreen cognitive sign-off timestamp (pilot)</t>
+  </si>
+  <si>
+    <t>Touchscreen sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Urine collection sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Verbal nterview sign-off timestamp</t>
+  </si>
+  <si>
+    <t>Blood sample #, note contents</t>
+  </si>
+  <si>
+    <t>Reason blood sampling not attempted</t>
+  </si>
+  <si>
+    <t>Was blood sampling attempted</t>
+  </si>
+  <si>
+    <t>Number of blood samples taken</t>
+  </si>
+  <si>
+    <t>Time blood sample collected</t>
+  </si>
+  <si>
+    <t>Fasting time</t>
   </si>
 </sst>
 </file>
@@ -487,12 +590,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -508,7 +617,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -534,6 +643,9 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1000,6 +1112,385 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB0D2D7A-D1F6-4EF1-89BA-0683EFCB5A9A}">
+  <dimension ref="A1:F48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="15">
+        <v>3166</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="15">
+        <v>21834</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="15">
+        <v>21871</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="15">
+        <v>21862</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="15">
+        <v>21865</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="15">
+        <v>21863</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="15">
+        <v>21851</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="15">
+        <v>21821</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="15">
+        <v>21864</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="15">
+        <v>21866</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="15">
+        <v>21838</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="15">
+        <v>21836</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="15">
+        <v>21861</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="15">
+        <v>21833</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="15">
+        <v>21832</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="15">
+        <v>21811</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="15">
+        <v>21842</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="15">
+        <v>21825</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="15">
+        <v>21823</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="15">
+        <v>21822</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="15">
+        <v>21841</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="15">
+        <v>21831</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="15">
+        <v>20049</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="15">
+        <v>20050</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="15">
+        <v>35</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="15">
+        <v>68</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="15">
+        <v>74</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="15">
+        <v>4</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="15">
+        <v>6</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="15">
+        <v>6022</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="15">
+        <v>5198</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="15">
+        <v>5</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="15">
+        <v>630</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="15">
+        <v>3</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A42" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=4" xr:uid="{C945E10A-2AF1-44D5-B6C3-5BB9C76FA051}"/>
+    <hyperlink ref="B42" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=4" xr:uid="{F8F062EB-6094-4B7B-A02B-9F95719D500D}"/>
+    <hyperlink ref="A43" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=6" xr:uid="{C7A85AA4-347B-4FAC-A09B-9A84B40C321B}"/>
+    <hyperlink ref="B43" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=6" xr:uid="{C5FFC46F-FD4B-48A5-8C16-17EDCF68711A}"/>
+    <hyperlink ref="A44" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=6022" xr:uid="{559F676B-EA61-4E93-A63C-57C702733208}"/>
+    <hyperlink ref="B44" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=6022" xr:uid="{09789168-C385-4E4C-B7CF-A845B76C8B86}"/>
+    <hyperlink ref="A45" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=5198" xr:uid="{2C1E0CC6-8A30-4762-A7FB-97C54C60E98A}"/>
+    <hyperlink ref="B45" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=5198" xr:uid="{5D6F8ACC-CEE9-485B-89C4-D66FC34E2984}"/>
+    <hyperlink ref="A46" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=5" xr:uid="{2E83B23F-CBDC-45CD-A5CE-63364D0CFB0F}"/>
+    <hyperlink ref="B46" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=5" xr:uid="{6DA1A3DC-50FE-45EF-AFB3-022A52EC5943}"/>
+    <hyperlink ref="A47" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=630" xr:uid="{7DE4487C-B523-4091-8E95-AC31C1A1404F}"/>
+    <hyperlink ref="B47" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=630" xr:uid="{C8CF3640-C99B-443A-AE1F-BF27719E9A11}"/>
+    <hyperlink ref="A48" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3" xr:uid="{A8D9C800-C7D1-456A-A7E9-DFA80A0F32F3}"/>
+    <hyperlink ref="B48" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3" xr:uid="{43E7E12B-1265-4115-8008-3A2A88FF31D4}"/>
+    <hyperlink ref="A3" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21834" xr:uid="{526B15D3-112B-428C-8147-6F48C0BF65B1}"/>
+    <hyperlink ref="B3" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21834" xr:uid="{14257988-9914-4BFB-BEF8-D7EBBC35CF10}"/>
+    <hyperlink ref="A14" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21862" xr:uid="{2FD4A2EB-3822-460B-9495-C4FCC376A7F4}"/>
+    <hyperlink ref="B14" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21862" xr:uid="{F058C6AF-668F-4E93-ADA9-C9507721140B}"/>
+    <hyperlink ref="A4" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21871" xr:uid="{C9C951AA-0217-414F-983E-B525AE3E7CE7}"/>
+    <hyperlink ref="B4" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21871" xr:uid="{D08DF806-AB73-4346-BF76-89168F47CC15}"/>
+    <hyperlink ref="A16" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21865" xr:uid="{E060783D-CB52-4481-AEA9-1BD653A5C1FA}"/>
+    <hyperlink ref="B16" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21865" xr:uid="{C2E6BD00-9367-4DA3-8D52-421A0D7C4B10}"/>
+    <hyperlink ref="A17" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21863" xr:uid="{D055A164-9A30-4CF4-9F3E-8B327247BA08}"/>
+    <hyperlink ref="B17" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21863" xr:uid="{1B03A119-64FC-42C9-BE19-8CEA28AE167A}"/>
+    <hyperlink ref="A18" r:id="rId25" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21851" xr:uid="{1BAEAD3F-E910-4E9B-B5EA-9F8CBA09E20C}"/>
+    <hyperlink ref="B18" r:id="rId26" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21851" xr:uid="{EA928646-B216-4024-803B-8E8BEB449D81}"/>
+    <hyperlink ref="A19" r:id="rId27" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21821" xr:uid="{8DFD7B11-4560-4CE5-8CCB-2D5AE3560126}"/>
+    <hyperlink ref="B19" r:id="rId28" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21821" xr:uid="{3A290BA0-7819-439F-B039-8D2FD5AF8C47}"/>
+    <hyperlink ref="A20" r:id="rId29" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21864" xr:uid="{B95545F8-19C7-4332-B835-A32BBD9F57EF}"/>
+    <hyperlink ref="B20" r:id="rId30" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21864" xr:uid="{C08A6346-6511-4214-B35A-BE81D820D5B5}"/>
+    <hyperlink ref="A21" r:id="rId31" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21866" xr:uid="{C9FEF6B7-A5CD-48C6-9865-AC0645EDA4F3}"/>
+    <hyperlink ref="B21" r:id="rId32" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21866" xr:uid="{FEF51254-A330-4FA5-8537-D903C1938803}"/>
+    <hyperlink ref="A22" r:id="rId33" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21838" xr:uid="{0945E04C-45B3-474D-B512-0ACCFAB3D497}"/>
+    <hyperlink ref="B22" r:id="rId34" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21838" xr:uid="{5ADCDC39-B12F-426C-B90F-235FBC82EF88}"/>
+    <hyperlink ref="A23" r:id="rId35" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21836" xr:uid="{3928CAC3-7619-45E7-8422-376372B67C07}"/>
+    <hyperlink ref="B23" r:id="rId36" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21836" xr:uid="{0051965A-D761-4543-98F7-14514B7CA2A7}"/>
+    <hyperlink ref="A24" r:id="rId37" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21861" xr:uid="{3BBBA7C4-1DFD-4148-95DF-D917DA38A386}"/>
+    <hyperlink ref="B24" r:id="rId38" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21861" xr:uid="{05FEA658-5F5E-415D-A4B9-435F2B68EAF8}"/>
+    <hyperlink ref="A25" r:id="rId39" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21833" xr:uid="{BA43D26A-68D0-485B-B6B4-04B19D8A896F}"/>
+    <hyperlink ref="B25" r:id="rId40" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21833" xr:uid="{5C7C4266-2173-43FE-8C39-6FF50667D48D}"/>
+    <hyperlink ref="A26" r:id="rId41" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21832" xr:uid="{6EACE88F-B87E-4CC2-8FB7-A3C450CC4461}"/>
+    <hyperlink ref="B26" r:id="rId42" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21832" xr:uid="{5C3315D4-AED1-4A02-BDB0-3139B636A510}"/>
+    <hyperlink ref="A27" r:id="rId43" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21811" xr:uid="{DD282F5A-B7DC-4E91-A56E-2E27D68ACB0F}"/>
+    <hyperlink ref="B27" r:id="rId44" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21811" xr:uid="{995FD4B3-59D9-45D0-B950-AE76EEA9CAB8}"/>
+    <hyperlink ref="A28" r:id="rId45" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21842" xr:uid="{57D72DDA-75E3-4658-A808-7A05FA0DCDA6}"/>
+    <hyperlink ref="B28" r:id="rId46" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21842" xr:uid="{FFB9D9D1-145F-43D2-B8EF-7B385E877BE0}"/>
+    <hyperlink ref="A29" r:id="rId47" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21825" xr:uid="{B4F6C5BF-CA74-4083-97E8-57384888E7B3}"/>
+    <hyperlink ref="B29" r:id="rId48" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21825" xr:uid="{D002667E-9A41-4DE0-8899-2D861B217202}"/>
+    <hyperlink ref="A30" r:id="rId49" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21823" xr:uid="{3ED9711F-20DD-4FC7-BB96-B6E9A8AF496A}"/>
+    <hyperlink ref="B30" r:id="rId50" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21823" xr:uid="{A98D9E6F-0F00-4F8F-BF7E-C1854B70994A}"/>
+    <hyperlink ref="A31" r:id="rId51" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21822" xr:uid="{90BA2A6C-D099-41CC-9778-B592287EB7BD}"/>
+    <hyperlink ref="B31" r:id="rId52" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21822" xr:uid="{583C3707-D780-42CD-9867-99CF9D92191F}"/>
+    <hyperlink ref="A32" r:id="rId53" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21841" xr:uid="{729E4DD7-07AD-4EA7-9D7E-76B6AE9607CF}"/>
+    <hyperlink ref="B32" r:id="rId54" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21841" xr:uid="{CA975996-50CF-480C-9AB2-92F048F9E25C}"/>
+    <hyperlink ref="A33" r:id="rId55" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21831" xr:uid="{0CD2E893-254A-41E5-9A06-531A32BDF7A9}"/>
+    <hyperlink ref="B33" r:id="rId56" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21831" xr:uid="{39FF6F7F-2C03-4C70-A2E2-444EC49D1E62}"/>
+    <hyperlink ref="A35" r:id="rId57" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=20049" xr:uid="{90B4DC71-6F3F-481E-92F1-5686BCBBA618}"/>
+    <hyperlink ref="B35" r:id="rId58" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=20049" xr:uid="{E99C73FB-E128-447D-9B45-C280B1176622}"/>
+    <hyperlink ref="A36" r:id="rId59" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=20050" xr:uid="{32346BA6-86D6-4FE0-8BCD-D6B9F09D182F}"/>
+    <hyperlink ref="B36" r:id="rId60" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=20050" xr:uid="{EF0EA3D1-975A-43D9-A50E-70C746E6A42C}"/>
+    <hyperlink ref="A37" r:id="rId61" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=35" xr:uid="{D86D60A3-72ED-4005-981E-C8FCDC803F98}"/>
+    <hyperlink ref="B37" r:id="rId62" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=35" xr:uid="{95B10406-7624-4536-9831-E2528766CCDB}"/>
+    <hyperlink ref="A38" r:id="rId63" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=68" xr:uid="{2C1AE4DC-F069-4F36-B622-C06665FAAA4D}"/>
+    <hyperlink ref="B38" r:id="rId64" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=68" xr:uid="{7464F8C7-8045-43C3-851D-54B664D9F4CD}"/>
+    <hyperlink ref="A2" r:id="rId65" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3166" xr:uid="{2E54CEF5-EB08-4252-B948-77997BA30409}"/>
+    <hyperlink ref="B2" r:id="rId66" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3166" xr:uid="{696FC014-5D06-4B96-87DF-3F5F6FC8F032}"/>
+    <hyperlink ref="A40" r:id="rId67" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=74" xr:uid="{329612AF-7F04-4213-A8F1-B675AC9B2F23}"/>
+    <hyperlink ref="B40" r:id="rId68" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=74" xr:uid="{0B82E0E8-5E5F-480D-82B8-1ADD68C0D437}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId69"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F3"/>
@@ -2453,11 +2944,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2676,27 +3168,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2721,9 +3203,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated core_vars_data_dict to include derived variables
</commit_message>
<xml_diff>
--- a/Get variables/core_var_data_dict.xlsx
+++ b/Get variables/core_var_data_dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arogusk2\OneDrive - University of Edinburgh\HELIOS-BD\Side Projects\BioBank Project\Git\biobank-time-dimensions\Get variables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B437E2A0-61B2-44D4-AF16-8B33579B967B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE1FCE96-DB2D-4083-A3CB-5BF85907C611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1875" windowWidth="29040" windowHeight="15840" tabRatio="849" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1875" windowWidth="29040" windowHeight="15840" tabRatio="849" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Primary demographics" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,8 @@
     <sheet name="Seasonal" sheetId="13" r:id="rId7"/>
     <sheet name="Sleep" sheetId="10" r:id="rId8"/>
     <sheet name="Physical measure summary" sheetId="3" r:id="rId9"/>
-    <sheet name="Data Collection Timings" sheetId="14" r:id="rId10"/>
+    <sheet name="Photoperiod vars" sheetId="15" r:id="rId10"/>
+    <sheet name="Data Collection Timings" sheetId="14" r:id="rId11"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="206">
   <si>
     <t>General health  </t>
   </si>
@@ -459,42 +460,15 @@
     <t>alcohol_yesterday</t>
   </si>
   <si>
-    <t>Biometrics duration</t>
-  </si>
-  <si>
-    <t>Conclusion duration</t>
-  </si>
-  <si>
-    <t>ECG during exercise duration</t>
-  </si>
-  <si>
-    <t>Eye measures duration</t>
-  </si>
-  <si>
-    <t>Sample collection duration</t>
-  </si>
-  <si>
-    <t>Touchscreen duration</t>
-  </si>
-  <si>
-    <t>Verbal interview duration</t>
-  </si>
-  <si>
     <t>Biometrics sign-off timestamp</t>
   </si>
   <si>
-    <t>Brain MRI sign-off timestamp</t>
-  </si>
-  <si>
     <t>Cardiac monitor sign-off timestamp</t>
   </si>
   <si>
     <t>Carotid ultrasound sign-off timestamp</t>
   </si>
   <si>
-    <t>Chest MRI sign-off timestamp</t>
-  </si>
-  <si>
     <t>Conclusion sign-off timestamp</t>
   </si>
   <si>
@@ -513,15 +487,6 @@
     <t>Eye measures sign-off timestamp</t>
   </si>
   <si>
-    <t>Imaging screening sign-off timestamp</t>
-  </si>
-  <si>
-    <t>Measurement/Impedance sign-off timestamp (pilot)</t>
-  </si>
-  <si>
-    <t>Pilot Spirometry sign-off timestamp</t>
-  </si>
-  <si>
     <t>Reception sign-off timestamp</t>
   </si>
   <si>
@@ -531,9 +496,6 @@
     <t>Touchscreen cognitive sign-off timestamp</t>
   </si>
   <si>
-    <t>Touchscreen cognitive sign-off timestamp (pilot)</t>
-  </si>
-  <si>
     <t>Touchscreen sign-off timestamp</t>
   </si>
   <si>
@@ -543,29 +505,161 @@
     <t>Verbal nterview sign-off timestamp</t>
   </si>
   <si>
-    <t>Blood sample #, note contents</t>
-  </si>
-  <si>
-    <t>Reason blood sampling not attempted</t>
-  </si>
-  <si>
-    <t>Was blood sampling attempted</t>
-  </si>
-  <si>
-    <t>Number of blood samples taken</t>
-  </si>
-  <si>
     <t>Time blood sample collected</t>
   </si>
   <si>
-    <t>Fasting time</t>
+    <t>BS_time</t>
+  </si>
+  <si>
+    <t>end_biometrics</t>
+  </si>
+  <si>
+    <t>end_consent</t>
+  </si>
+  <si>
+    <t>end_reception</t>
+  </si>
+  <si>
+    <t>end_touchscreen</t>
+  </si>
+  <si>
+    <t>end_cardiac</t>
+  </si>
+  <si>
+    <t>end_carotid</t>
+  </si>
+  <si>
+    <t>end_dxa</t>
+  </si>
+  <si>
+    <t>end_ecg</t>
+  </si>
+  <si>
+    <t>end_eye</t>
+  </si>
+  <si>
+    <t>end_sample</t>
+  </si>
+  <si>
+    <t>end_urine</t>
+  </si>
+  <si>
+    <t>end_signoff</t>
+  </si>
+  <si>
+    <t>end_ecg_exercise</t>
+  </si>
+  <si>
+    <t>end_touchscreen_cog</t>
+  </si>
+  <si>
+    <t>end_interview</t>
+  </si>
+  <si>
+    <t>derived</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>Month of attending assessment centre</t>
+  </si>
+  <si>
+    <t>Year of attending assessment centre</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>Time of blood sample</t>
+  </si>
+  <si>
+    <t>BS_month</t>
+  </si>
+  <si>
+    <t>Month of blood sample</t>
+  </si>
+  <si>
+    <t>derived from 53</t>
+  </si>
+  <si>
+    <t>derived from 3166</t>
+  </si>
+  <si>
+    <t>derived field</t>
+  </si>
+  <si>
+    <t>Assessment centre latitude</t>
+  </si>
+  <si>
+    <t>Assessment centre longitude</t>
+  </si>
+  <si>
+    <t>Assessment centre name</t>
+  </si>
+  <si>
+    <t>assess_name</t>
+  </si>
+  <si>
+    <t>assess_latitude</t>
+  </si>
+  <si>
+    <t>assess_longitude</t>
+  </si>
+  <si>
+    <t>julian_day</t>
+  </si>
+  <si>
+    <t>prev_julian_day</t>
+  </si>
+  <si>
+    <t>daylength_min</t>
+  </si>
+  <si>
+    <t>prev_daylength_min</t>
+  </si>
+  <si>
+    <t>photoperiod_roc_min</t>
+  </si>
+  <si>
+    <t>photoperiod_roc_percent</t>
+  </si>
+  <si>
+    <t>Julian day date</t>
+  </si>
+  <si>
+    <t>Previous day's Julian day date</t>
+  </si>
+  <si>
+    <t>derived from 54</t>
+  </si>
+  <si>
+    <t>derived from 55</t>
+  </si>
+  <si>
+    <t>derived from 56</t>
+  </si>
+  <si>
+    <t>Daylength on assessment date</t>
+  </si>
+  <si>
+    <t>Daylength on day prior to assessment date</t>
+  </si>
+  <si>
+    <t>Photoperiod rate of change between previous dat &amp; assessment day (minutes)</t>
+  </si>
+  <si>
+    <t>Photoperiod rate of change between previous dat &amp; assessment day (percentage)</t>
+  </si>
+  <si>
+    <t>/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -589,19 +683,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -617,7 +725,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -643,9 +751,10 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1113,387 +1222,866 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB0D2D7A-D1F6-4EF1-89BA-0683EFCB5A9A}">
-  <dimension ref="A1:F48"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3BE1359-67D3-4700-9D16-53E4747F7CC2}">
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="2" max="2" width="62.5703125" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C3" t="s">
+        <v>205</v>
+      </c>
+      <c r="D3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C4" t="s">
+        <v>205</v>
+      </c>
+      <c r="D4" t="s">
+        <v>192</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>200</v>
+      </c>
+      <c r="B5" t="s">
+        <v>202</v>
+      </c>
+      <c r="C5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D6" t="s">
+        <v>194</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>173</v>
+      </c>
+      <c r="B7" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" t="s">
+        <v>205</v>
+      </c>
+      <c r="D7" t="s">
+        <v>195</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C8" s="16"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C9" s="16"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB0D2D7A-D1F6-4EF1-89BA-0683EFCB5A9A}">
+  <dimension ref="A1:G52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="25.28515625" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="10" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="15">
+    <row r="2" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="11">
         <v>3166</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="15">
+      <c r="B2" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="11">
         <v>21834</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11">
+        <v>21871</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="11">
+        <v>21865</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11">
+        <v>21851</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11">
+        <v>21821</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="11">
+        <v>21864</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="11">
+        <v>21866</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11">
+        <v>21838</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
-        <v>21871</v>
-      </c>
-      <c r="B4" s="15" t="s">
+      <c r="D10" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="11">
+        <v>21836</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11">
+        <v>21811</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
-        <v>21862</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
-        <v>21865</v>
-      </c>
-      <c r="B16" s="15" t="s">
+      <c r="D12" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="11">
+        <v>21842</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
-        <v>21863</v>
-      </c>
-      <c r="B17" s="15" t="s">
+      <c r="D13" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="11">
+        <v>21825</v>
+      </c>
+      <c r="B14" s="11" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
-        <v>21851</v>
+      <c r="D14" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="11">
+        <v>21822</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="11">
+        <v>21841</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="11">
+        <v>21831</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" t="s">
+        <v>181</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
-        <v>21821</v>
+        <v>175</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>181</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
-        <v>21864</v>
+        <v>176</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
+        <v>182</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
-        <v>21866</v>
+        <v>178</v>
+      </c>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F20" t="s">
+        <v>75</v>
+      </c>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
+        <v>182</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
-        <v>21838</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
-        <v>21836</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
-        <v>21861</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
-        <v>21833</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="15">
-        <v>21832</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
-        <v>21811</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="15">
-        <v>21842</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
-        <v>21825</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="15">
-        <v>21823</v>
-      </c>
-      <c r="B30" s="15" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="15">
-        <v>21822</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="15">
-        <v>21841</v>
-      </c>
-      <c r="B32" s="15" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
-        <v>21831</v>
-      </c>
-      <c r="B33" s="15" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="15">
-        <v>20049</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="15">
-        <v>20050</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="15">
-        <v>35</v>
-      </c>
-      <c r="B37" s="15" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="15">
-        <v>68</v>
-      </c>
-      <c r="B38" s="15" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="15">
-        <v>74</v>
-      </c>
-      <c r="B40" s="15" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="15">
-        <v>4</v>
-      </c>
-      <c r="B42" s="15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="15">
-        <v>6</v>
-      </c>
-      <c r="B43" s="15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="15">
-        <v>6022</v>
-      </c>
-      <c r="B44" s="15" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="15">
-        <v>5198</v>
-      </c>
-      <c r="B45" s="15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="15">
-        <v>5</v>
-      </c>
-      <c r="B46" s="15" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="15">
-        <v>630</v>
-      </c>
-      <c r="B47" s="15" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="15">
-        <v>3</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>147</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F21" t="s">
+        <v>75</v>
+      </c>
+      <c r="G21" s="10"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="11"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="11"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="10"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="10"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="10"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="11"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="10"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="10"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="10"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="10"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="11"/>
+      <c r="B37" s="11"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="11"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="11"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="10"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="11"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="10"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="11"/>
+      <c r="B43" s="11"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="11"/>
+      <c r="B44" s="11"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="11"/>
+      <c r="B45" s="11"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="11"/>
+      <c r="B46" s="11"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="11"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="11"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="11"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="10"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="10"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="10"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="10"/>
+      <c r="G52" s="10"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A42" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=4" xr:uid="{C945E10A-2AF1-44D5-B6C3-5BB9C76FA051}"/>
-    <hyperlink ref="B42" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=4" xr:uid="{F8F062EB-6094-4B7B-A02B-9F95719D500D}"/>
-    <hyperlink ref="A43" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=6" xr:uid="{C7A85AA4-347B-4FAC-A09B-9A84B40C321B}"/>
-    <hyperlink ref="B43" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=6" xr:uid="{C5FFC46F-FD4B-48A5-8C16-17EDCF68711A}"/>
-    <hyperlink ref="A44" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=6022" xr:uid="{559F676B-EA61-4E93-A63C-57C702733208}"/>
-    <hyperlink ref="B44" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=6022" xr:uid="{09789168-C385-4E4C-B7CF-A845B76C8B86}"/>
-    <hyperlink ref="A45" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=5198" xr:uid="{2C1E0CC6-8A30-4762-A7FB-97C54C60E98A}"/>
-    <hyperlink ref="B45" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=5198" xr:uid="{5D6F8ACC-CEE9-485B-89C4-D66FC34E2984}"/>
-    <hyperlink ref="A46" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=5" xr:uid="{2E83B23F-CBDC-45CD-A5CE-63364D0CFB0F}"/>
-    <hyperlink ref="B46" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=5" xr:uid="{6DA1A3DC-50FE-45EF-AFB3-022A52EC5943}"/>
-    <hyperlink ref="A47" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=630" xr:uid="{7DE4487C-B523-4091-8E95-AC31C1A1404F}"/>
-    <hyperlink ref="B47" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=630" xr:uid="{C8CF3640-C99B-443A-AE1F-BF27719E9A11}"/>
-    <hyperlink ref="A48" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3" xr:uid="{A8D9C800-C7D1-456A-A7E9-DFA80A0F32F3}"/>
-    <hyperlink ref="B48" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3" xr:uid="{43E7E12B-1265-4115-8008-3A2A88FF31D4}"/>
-    <hyperlink ref="A3" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21834" xr:uid="{526B15D3-112B-428C-8147-6F48C0BF65B1}"/>
-    <hyperlink ref="B3" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21834" xr:uid="{14257988-9914-4BFB-BEF8-D7EBBC35CF10}"/>
-    <hyperlink ref="A14" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21862" xr:uid="{2FD4A2EB-3822-460B-9495-C4FCC376A7F4}"/>
-    <hyperlink ref="B14" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21862" xr:uid="{F058C6AF-668F-4E93-ADA9-C9507721140B}"/>
-    <hyperlink ref="A4" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21871" xr:uid="{C9C951AA-0217-414F-983E-B525AE3E7CE7}"/>
-    <hyperlink ref="B4" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21871" xr:uid="{D08DF806-AB73-4346-BF76-89168F47CC15}"/>
-    <hyperlink ref="A16" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21865" xr:uid="{E060783D-CB52-4481-AEA9-1BD653A5C1FA}"/>
-    <hyperlink ref="B16" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21865" xr:uid="{C2E6BD00-9367-4DA3-8D52-421A0D7C4B10}"/>
-    <hyperlink ref="A17" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21863" xr:uid="{D055A164-9A30-4CF4-9F3E-8B327247BA08}"/>
-    <hyperlink ref="B17" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21863" xr:uid="{1B03A119-64FC-42C9-BE19-8CEA28AE167A}"/>
-    <hyperlink ref="A18" r:id="rId25" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21851" xr:uid="{1BAEAD3F-E910-4E9B-B5EA-9F8CBA09E20C}"/>
-    <hyperlink ref="B18" r:id="rId26" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21851" xr:uid="{EA928646-B216-4024-803B-8E8BEB449D81}"/>
-    <hyperlink ref="A19" r:id="rId27" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21821" xr:uid="{8DFD7B11-4560-4CE5-8CCB-2D5AE3560126}"/>
-    <hyperlink ref="B19" r:id="rId28" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21821" xr:uid="{3A290BA0-7819-439F-B039-8D2FD5AF8C47}"/>
-    <hyperlink ref="A20" r:id="rId29" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21864" xr:uid="{B95545F8-19C7-4332-B835-A32BBD9F57EF}"/>
-    <hyperlink ref="B20" r:id="rId30" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21864" xr:uid="{C08A6346-6511-4214-B35A-BE81D820D5B5}"/>
-    <hyperlink ref="A21" r:id="rId31" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21866" xr:uid="{C9FEF6B7-A5CD-48C6-9865-AC0645EDA4F3}"/>
-    <hyperlink ref="B21" r:id="rId32" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21866" xr:uid="{FEF51254-A330-4FA5-8537-D903C1938803}"/>
-    <hyperlink ref="A22" r:id="rId33" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21838" xr:uid="{0945E04C-45B3-474D-B512-0ACCFAB3D497}"/>
-    <hyperlink ref="B22" r:id="rId34" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21838" xr:uid="{5ADCDC39-B12F-426C-B90F-235FBC82EF88}"/>
-    <hyperlink ref="A23" r:id="rId35" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21836" xr:uid="{3928CAC3-7619-45E7-8422-376372B67C07}"/>
-    <hyperlink ref="B23" r:id="rId36" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21836" xr:uid="{0051965A-D761-4543-98F7-14514B7CA2A7}"/>
-    <hyperlink ref="A24" r:id="rId37" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21861" xr:uid="{3BBBA7C4-1DFD-4148-95DF-D917DA38A386}"/>
-    <hyperlink ref="B24" r:id="rId38" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21861" xr:uid="{05FEA658-5F5E-415D-A4B9-435F2B68EAF8}"/>
-    <hyperlink ref="A25" r:id="rId39" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21833" xr:uid="{BA43D26A-68D0-485B-B6B4-04B19D8A896F}"/>
-    <hyperlink ref="B25" r:id="rId40" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21833" xr:uid="{5C7C4266-2173-43FE-8C39-6FF50667D48D}"/>
-    <hyperlink ref="A26" r:id="rId41" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21832" xr:uid="{6EACE88F-B87E-4CC2-8FB7-A3C450CC4461}"/>
-    <hyperlink ref="B26" r:id="rId42" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21832" xr:uid="{5C3315D4-AED1-4A02-BDB0-3139B636A510}"/>
-    <hyperlink ref="A27" r:id="rId43" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21811" xr:uid="{DD282F5A-B7DC-4E91-A56E-2E27D68ACB0F}"/>
-    <hyperlink ref="B27" r:id="rId44" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21811" xr:uid="{995FD4B3-59D9-45D0-B950-AE76EEA9CAB8}"/>
-    <hyperlink ref="A28" r:id="rId45" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21842" xr:uid="{57D72DDA-75E3-4658-A808-7A05FA0DCDA6}"/>
-    <hyperlink ref="B28" r:id="rId46" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21842" xr:uid="{FFB9D9D1-145F-43D2-B8EF-7B385E877BE0}"/>
-    <hyperlink ref="A29" r:id="rId47" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21825" xr:uid="{B4F6C5BF-CA74-4083-97E8-57384888E7B3}"/>
-    <hyperlink ref="B29" r:id="rId48" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21825" xr:uid="{D002667E-9A41-4DE0-8899-2D861B217202}"/>
-    <hyperlink ref="A30" r:id="rId49" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21823" xr:uid="{3ED9711F-20DD-4FC7-BB96-B6E9A8AF496A}"/>
-    <hyperlink ref="B30" r:id="rId50" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21823" xr:uid="{A98D9E6F-0F00-4F8F-BF7E-C1854B70994A}"/>
-    <hyperlink ref="A31" r:id="rId51" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21822" xr:uid="{90BA2A6C-D099-41CC-9778-B592287EB7BD}"/>
-    <hyperlink ref="B31" r:id="rId52" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21822" xr:uid="{583C3707-D780-42CD-9867-99CF9D92191F}"/>
-    <hyperlink ref="A32" r:id="rId53" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21841" xr:uid="{729E4DD7-07AD-4EA7-9D7E-76B6AE9607CF}"/>
-    <hyperlink ref="B32" r:id="rId54" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21841" xr:uid="{CA975996-50CF-480C-9AB2-92F048F9E25C}"/>
-    <hyperlink ref="A33" r:id="rId55" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21831" xr:uid="{0CD2E893-254A-41E5-9A06-531A32BDF7A9}"/>
-    <hyperlink ref="B33" r:id="rId56" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21831" xr:uid="{39FF6F7F-2C03-4C70-A2E2-444EC49D1E62}"/>
-    <hyperlink ref="A35" r:id="rId57" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=20049" xr:uid="{90B4DC71-6F3F-481E-92F1-5686BCBBA618}"/>
-    <hyperlink ref="B35" r:id="rId58" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=20049" xr:uid="{E99C73FB-E128-447D-9B45-C280B1176622}"/>
-    <hyperlink ref="A36" r:id="rId59" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=20050" xr:uid="{32346BA6-86D6-4FE0-8BCD-D6B9F09D182F}"/>
-    <hyperlink ref="B36" r:id="rId60" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=20050" xr:uid="{EF0EA3D1-975A-43D9-A50E-70C746E6A42C}"/>
-    <hyperlink ref="A37" r:id="rId61" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=35" xr:uid="{D86D60A3-72ED-4005-981E-C8FCDC803F98}"/>
-    <hyperlink ref="B37" r:id="rId62" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=35" xr:uid="{95B10406-7624-4536-9831-E2528766CCDB}"/>
-    <hyperlink ref="A38" r:id="rId63" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=68" xr:uid="{2C1AE4DC-F069-4F36-B622-C06665FAAA4D}"/>
-    <hyperlink ref="B38" r:id="rId64" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=68" xr:uid="{7464F8C7-8045-43C3-851D-54B664D9F4CD}"/>
-    <hyperlink ref="A2" r:id="rId65" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3166" xr:uid="{2E54CEF5-EB08-4252-B948-77997BA30409}"/>
-    <hyperlink ref="B2" r:id="rId66" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3166" xr:uid="{696FC014-5D06-4B96-87DF-3F5F6FC8F032}"/>
-    <hyperlink ref="A40" r:id="rId67" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=74" xr:uid="{329612AF-7F04-4213-A8F1-B675AC9B2F23}"/>
-    <hyperlink ref="B40" r:id="rId68" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=74" xr:uid="{0B82E0E8-5E5F-480D-82B8-1ADD68C0D437}"/>
+    <hyperlink ref="A3" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21834" xr:uid="{526B15D3-112B-428C-8147-6F48C0BF65B1}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21834" xr:uid="{14257988-9914-4BFB-BEF8-D7EBBC35CF10}"/>
+    <hyperlink ref="A4" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21871" xr:uid="{C9C951AA-0217-414F-983E-B525AE3E7CE7}"/>
+    <hyperlink ref="B4" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21871" xr:uid="{D08DF806-AB73-4346-BF76-89168F47CC15}"/>
+    <hyperlink ref="A5" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21865" xr:uid="{E060783D-CB52-4481-AEA9-1BD653A5C1FA}"/>
+    <hyperlink ref="B5" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21865" xr:uid="{C2E6BD00-9367-4DA3-8D52-421A0D7C4B10}"/>
+    <hyperlink ref="A6" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21851" xr:uid="{1BAEAD3F-E910-4E9B-B5EA-9F8CBA09E20C}"/>
+    <hyperlink ref="B6" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21851" xr:uid="{EA928646-B216-4024-803B-8E8BEB449D81}"/>
+    <hyperlink ref="A7" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21821" xr:uid="{8DFD7B11-4560-4CE5-8CCB-2D5AE3560126}"/>
+    <hyperlink ref="B7" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21821" xr:uid="{3A290BA0-7819-439F-B039-8D2FD5AF8C47}"/>
+    <hyperlink ref="A8" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21864" xr:uid="{B95545F8-19C7-4332-B835-A32BBD9F57EF}"/>
+    <hyperlink ref="B8" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21864" xr:uid="{C08A6346-6511-4214-B35A-BE81D820D5B5}"/>
+    <hyperlink ref="A9" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21866" xr:uid="{C9FEF6B7-A5CD-48C6-9865-AC0645EDA4F3}"/>
+    <hyperlink ref="B9" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21866" xr:uid="{FEF51254-A330-4FA5-8537-D903C1938803}"/>
+    <hyperlink ref="A10" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21838" xr:uid="{0945E04C-45B3-474D-B512-0ACCFAB3D497}"/>
+    <hyperlink ref="B10" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21838" xr:uid="{5ADCDC39-B12F-426C-B90F-235FBC82EF88}"/>
+    <hyperlink ref="A11" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21836" xr:uid="{3928CAC3-7619-45E7-8422-376372B67C07}"/>
+    <hyperlink ref="B11" r:id="rId18" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21836" xr:uid="{0051965A-D761-4543-98F7-14514B7CA2A7}"/>
+    <hyperlink ref="A12" r:id="rId19" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21811" xr:uid="{DD282F5A-B7DC-4E91-A56E-2E27D68ACB0F}"/>
+    <hyperlink ref="B12" r:id="rId20" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21811" xr:uid="{995FD4B3-59D9-45D0-B950-AE76EEA9CAB8}"/>
+    <hyperlink ref="A13" r:id="rId21" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21842" xr:uid="{57D72DDA-75E3-4658-A808-7A05FA0DCDA6}"/>
+    <hyperlink ref="B13" r:id="rId22" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21842" xr:uid="{FFB9D9D1-145F-43D2-B8EF-7B385E877BE0}"/>
+    <hyperlink ref="A14" r:id="rId23" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21825" xr:uid="{B4F6C5BF-CA74-4083-97E8-57384888E7B3}"/>
+    <hyperlink ref="B14" r:id="rId24" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21825" xr:uid="{D002667E-9A41-4DE0-8899-2D861B217202}"/>
+    <hyperlink ref="A15" r:id="rId25" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21822" xr:uid="{90BA2A6C-D099-41CC-9778-B592287EB7BD}"/>
+    <hyperlink ref="B15" r:id="rId26" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21822" xr:uid="{583C3707-D780-42CD-9867-99CF9D92191F}"/>
+    <hyperlink ref="A16" r:id="rId27" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21841" xr:uid="{729E4DD7-07AD-4EA7-9D7E-76B6AE9607CF}"/>
+    <hyperlink ref="B16" r:id="rId28" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21841" xr:uid="{CA975996-50CF-480C-9AB2-92F048F9E25C}"/>
+    <hyperlink ref="A17" r:id="rId29" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21831" xr:uid="{0CD2E893-254A-41E5-9A06-531A32BDF7A9}"/>
+    <hyperlink ref="B17" r:id="rId30" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=21831" xr:uid="{39FF6F7F-2C03-4C70-A2E2-444EC49D1E62}"/>
+    <hyperlink ref="A2" r:id="rId31" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3166" xr:uid="{2E54CEF5-EB08-4252-B948-77997BA30409}"/>
+    <hyperlink ref="B2" r:id="rId32" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?tk=AuGRRBvvOXrgxUmvX9MRYtILoVeOkW8d349824&amp;id=3166" xr:uid="{696FC014-5D06-4B96-87DF-3F5F6FC8F032}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId69"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId33"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="32.28515625" customWidth="1"/>
@@ -1560,6 +2148,57 @@
         <v>78</v>
       </c>
       <c r="F3" s="7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D5" t="s">
+        <v>188</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" t="s">
+        <v>189</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2944,12 +3583,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3168,17 +3806,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3203,18 +3851,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
added in basket info for var 3166 to check with cathy
</commit_message>
<xml_diff>
--- a/Get variables/core_var_data_dict.xlsx
+++ b/Get variables/core_var_data_dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arogusk2\OneDrive - University of Edinburgh\HELIOS-BD\Side Projects\BioBank Project\Git\biobank-time-dimensions\Get variables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE1FCE96-DB2D-4083-A3CB-5BF85907C611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{020E7E4A-A83E-41C7-9005-B7EE866F8949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1875" windowWidth="29040" windowHeight="15840" tabRatio="849" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="849" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Primary demographics" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="208">
   <si>
     <t>General health  </t>
   </si>
@@ -653,6 +653,12 @@
   </si>
   <si>
     <t>/</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>from basket 4066697</t>
   </si>
 </sst>
 </file>
@@ -1396,7 +1402,7 @@
     <col min="5" max="5" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>67</v>
       </c>
@@ -1415,8 +1421,11 @@
       <c r="F1" s="10" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G1" s="10" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11">
         <v>3166</v>
       </c>
@@ -1432,8 +1441,11 @@
       <c r="F2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G2" s="10" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
         <v>21834</v>
       </c>
@@ -1450,7 +1462,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11">
         <v>21871</v>
       </c>
@@ -1467,7 +1479,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11">
         <v>21865</v>
       </c>
@@ -1484,7 +1496,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11">
         <v>21851</v>
       </c>
@@ -1501,7 +1513,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11">
         <v>21821</v>
       </c>
@@ -1518,7 +1530,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11">
         <v>21864</v>
       </c>
@@ -1535,7 +1547,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
         <v>21866</v>
       </c>
@@ -1552,7 +1564,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
         <v>21838</v>
       </c>
@@ -1569,7 +1581,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
         <v>21836</v>
       </c>
@@ -1586,7 +1598,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
         <v>21811</v>
       </c>
@@ -1603,7 +1615,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
         <v>21842</v>
       </c>
@@ -1620,7 +1632,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
         <v>21825</v>
       </c>
@@ -1637,7 +1649,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11">
         <v>21822</v>
       </c>
@@ -1654,7 +1666,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
         <v>21841</v>
       </c>
@@ -3583,14 +3595,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002D5D40E36B58B0418A5C0DC6F6A2845B" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a816bc34d4292327d4a371c81c74c3a5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xmlns:ns4="301edac2-2a5a-4564-9129-5d780cc3d1d3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="773e6490813a0ac7eb54afe68e0456d4" ns3:_="" ns4:_="">
     <xsd:import namespace="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
@@ -3805,6 +3809,14 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3815,23 +3827,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD47ECBE-2CA4-4905-9B25-5B5DD8B09919}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3850,6 +3845,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
added weather variables to data dict
</commit_message>
<xml_diff>
--- a/Get variables/core_var_data_dict.xlsx
+++ b/Get variables/core_var_data_dict.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arogusk2\OneDrive - University of Edinburgh\HELIOS-BD\Side Projects\BioBank Project\Git\biobank-time-dimensions\Get variables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoe-my.sharepoint.com/personal/arogusk2_ed_ac_uk/Documents/HELIOS-BD/Side Projects/BioBank Project/Git/biobank-time-dimensions/Get variables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{020E7E4A-A83E-41C7-9005-B7EE866F8949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{020E7E4A-A83E-41C7-9005-B7EE866F8949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47DE2A81-B512-4A4D-9FA0-E940D9F54AF8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="849" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" tabRatio="849" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Primary demographics" sheetId="2" r:id="rId1"/>
@@ -20,10 +20,11 @@
     <sheet name="Early Life" sheetId="7" r:id="rId5"/>
     <sheet name="Health" sheetId="12" r:id="rId6"/>
     <sheet name="Seasonal" sheetId="13" r:id="rId7"/>
-    <sheet name="Sleep" sheetId="10" r:id="rId8"/>
-    <sheet name="Physical measure summary" sheetId="3" r:id="rId9"/>
+    <sheet name="Physical measure summary" sheetId="3" r:id="rId8"/>
+    <sheet name="Sleep" sheetId="10" r:id="rId9"/>
     <sheet name="Photoperiod vars" sheetId="15" r:id="rId10"/>
     <sheet name="Data Collection Timings" sheetId="14" r:id="rId11"/>
+    <sheet name="Weather" sheetId="16" r:id="rId12"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="223">
   <si>
     <t>General health  </t>
   </si>
@@ -659,6 +660,51 @@
   </si>
   <si>
     <t>from basket 4066697</t>
+  </si>
+  <si>
+    <t>station</t>
+  </si>
+  <si>
+    <t>tmax</t>
+  </si>
+  <si>
+    <t>tmin</t>
+  </si>
+  <si>
+    <t>frost</t>
+  </si>
+  <si>
+    <t>rain</t>
+  </si>
+  <si>
+    <t>sun</t>
+  </si>
+  <si>
+    <t>average_temp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">from CW weather script https://github.com/chronopsychiatry/biobank-time-dimensions/blob/main/Get%20variables/Get_weather_data.Rmd </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean daily maximum temperature (tmax)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean daily minimum temperature (tmin)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days of air frost (af)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total rainfall (rain)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total sunshine duration (sun)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly mean temperature  </t>
+  </si>
+  <si>
+    <t>closeast weather station to assessment centre</t>
   </si>
 </sst>
 </file>
@@ -1077,14 +1123,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="54.85546875" customWidth="1"/>
+    <col min="2" max="2" width="54.88671875" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" customWidth="1"/>
+    <col min="5" max="5" width="20.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -1104,7 +1150,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>31</v>
       </c>
@@ -1124,7 +1170,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>21003</v>
       </c>
@@ -1144,7 +1190,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>34</v>
       </c>
@@ -1164,7 +1210,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>52</v>
       </c>
@@ -1184,7 +1230,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>21000</v>
       </c>
@@ -1230,16 +1276,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3BE1359-67D3-4700-9D16-53E4747F7CC2}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="62.5703125" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="62.5546875" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -1259,7 +1305,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>181</v>
       </c>
@@ -1279,7 +1325,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>198</v>
       </c>
@@ -1299,7 +1345,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>199</v>
       </c>
@@ -1319,7 +1365,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>200</v>
       </c>
@@ -1339,7 +1385,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>173</v>
       </c>
@@ -1359,7 +1405,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>173</v>
       </c>
@@ -1379,10 +1425,10 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C8" s="16"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C9" s="16"/>
     </row>
   </sheetData>
@@ -1394,15 +1440,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB0D2D7A-D1F6-4EF1-89BA-0683EFCB5A9A}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="25.28515625" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="2" max="2" width="25.33203125" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>67</v>
       </c>
@@ -1425,7 +1471,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11">
         <v>3166</v>
       </c>
@@ -1445,7 +1491,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11">
         <v>21834</v>
       </c>
@@ -1462,7 +1508,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11">
         <v>21871</v>
       </c>
@@ -1479,7 +1525,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11">
         <v>21865</v>
       </c>
@@ -1496,7 +1542,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11">
         <v>21851</v>
       </c>
@@ -1513,7 +1559,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>21821</v>
       </c>
@@ -1530,7 +1576,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <v>21864</v>
       </c>
@@ -1547,7 +1593,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11">
         <v>21866</v>
       </c>
@@ -1564,7 +1610,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11">
         <v>21838</v>
       </c>
@@ -1581,7 +1627,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11">
         <v>21836</v>
       </c>
@@ -1598,7 +1644,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
         <v>21811</v>
       </c>
@@ -1615,7 +1661,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
         <v>21842</v>
       </c>
@@ -1632,7 +1678,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11">
         <v>21825</v>
       </c>
@@ -1649,7 +1695,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
         <v>21822</v>
       </c>
@@ -1666,7 +1712,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11">
         <v>21841</v>
       </c>
@@ -1683,7 +1729,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="17" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11">
         <v>21831</v>
       </c>
@@ -1700,7 +1746,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="15" t="s">
         <v>181</v>
       </c>
@@ -1717,7 +1763,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="15" t="s">
         <v>181</v>
       </c>
@@ -1734,7 +1780,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="15" t="s">
         <v>182</v>
       </c>
@@ -1753,7 +1799,7 @@
       </c>
       <c r="G20" s="10"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
         <v>182</v>
       </c>
@@ -1772,7 +1818,7 @@
       </c>
       <c r="G21" s="10"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -1781,7 +1827,7 @@
       <c r="F22" s="10"/>
       <c r="G22" s="10"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="10"/>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
@@ -1790,7 +1836,7 @@
       <c r="F23" s="10"/>
       <c r="G23" s="10"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -1799,7 +1845,7 @@
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="11"/>
       <c r="B25" s="11"/>
       <c r="C25" s="10"/>
@@ -1808,7 +1854,7 @@
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="11"/>
       <c r="B26" s="11"/>
       <c r="C26" s="10"/>
@@ -1817,7 +1863,7 @@
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="11"/>
       <c r="B27" s="11"/>
       <c r="C27" s="10"/>
@@ -1826,7 +1872,7 @@
       <c r="F27" s="10"/>
       <c r="G27" s="10"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -1835,7 +1881,7 @@
       <c r="F28" s="10"/>
       <c r="G28" s="10"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
@@ -1844,7 +1890,7 @@
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -1853,7 +1899,7 @@
       <c r="F30" s="10"/>
       <c r="G30" s="10"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="11"/>
       <c r="B31" s="11"/>
       <c r="C31" s="10"/>
@@ -1862,7 +1908,7 @@
       <c r="F31" s="10"/>
       <c r="G31" s="10"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
@@ -1871,7 +1917,7 @@
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
@@ -1880,7 +1926,7 @@
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
@@ -1889,7 +1935,7 @@
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -1898,7 +1944,7 @@
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="11"/>
       <c r="B36" s="11"/>
       <c r="C36" s="10"/>
@@ -1907,7 +1953,7 @@
       <c r="F36" s="10"/>
       <c r="G36" s="10"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="11"/>
       <c r="B37" s="11"/>
       <c r="C37" s="10"/>
@@ -1916,7 +1962,7 @@
       <c r="F37" s="10"/>
       <c r="G37" s="10"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="11"/>
       <c r="B38" s="11"/>
       <c r="C38" s="10"/>
@@ -1925,7 +1971,7 @@
       <c r="F38" s="10"/>
       <c r="G38" s="10"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="11"/>
       <c r="B39" s="11"/>
       <c r="C39" s="10"/>
@@ -1934,7 +1980,7 @@
       <c r="F39" s="10"/>
       <c r="G39" s="10"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="10"/>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
@@ -1943,7 +1989,7 @@
       <c r="F40" s="10"/>
       <c r="G40" s="10"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="11"/>
       <c r="B41" s="11"/>
       <c r="C41" s="10"/>
@@ -1952,7 +1998,7 @@
       <c r="F41" s="10"/>
       <c r="G41" s="10"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="10"/>
       <c r="B42" s="10"/>
       <c r="C42" s="10"/>
@@ -1961,7 +2007,7 @@
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="11"/>
       <c r="B43" s="11"/>
       <c r="C43" s="10"/>
@@ -1970,7 +2016,7 @@
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="11"/>
       <c r="B44" s="11"/>
       <c r="C44" s="10"/>
@@ -1979,7 +2025,7 @@
       <c r="F44" s="10"/>
       <c r="G44" s="10"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="11"/>
       <c r="B45" s="11"/>
       <c r="C45" s="10"/>
@@ -1988,7 +2034,7 @@
       <c r="F45" s="10"/>
       <c r="G45" s="10"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="11"/>
       <c r="B46" s="11"/>
       <c r="C46" s="10"/>
@@ -1997,7 +2043,7 @@
       <c r="F46" s="10"/>
       <c r="G46" s="10"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="11"/>
       <c r="B47" s="11"/>
       <c r="C47" s="10"/>
@@ -2006,7 +2052,7 @@
       <c r="F47" s="10"/>
       <c r="G47" s="10"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="11"/>
       <c r="B48" s="11"/>
       <c r="C48" s="10"/>
@@ -2015,7 +2061,7 @@
       <c r="F48" s="10"/>
       <c r="G48" s="10"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="11"/>
       <c r="B49" s="11"/>
       <c r="C49" s="10"/>
@@ -2024,7 +2070,7 @@
       <c r="F49" s="10"/>
       <c r="G49" s="10"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="10"/>
       <c r="B50" s="10"/>
       <c r="C50" s="10"/>
@@ -2033,7 +2079,7 @@
       <c r="F50" s="10"/>
       <c r="G50" s="10"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
@@ -2042,7 +2088,7 @@
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
@@ -2091,19 +2137,197 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CEAB4C2-B58D-40BE-890E-C58611A80C64}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="18.5546875" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3" t="s">
+        <v>216</v>
+      </c>
+      <c r="D3" t="s">
+        <v>209</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" t="s">
+        <v>120</v>
+      </c>
+      <c r="G3" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B4" t="s">
+        <v>217</v>
+      </c>
+      <c r="D4" t="s">
+        <v>210</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" t="s">
+        <v>120</v>
+      </c>
+      <c r="G4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" t="s">
+        <v>218</v>
+      </c>
+      <c r="D5" t="s">
+        <v>211</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" t="s">
+        <v>120</v>
+      </c>
+      <c r="G5" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D6" t="s">
+        <v>212</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
+        <v>120</v>
+      </c>
+      <c r="G6" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>173</v>
+      </c>
+      <c r="B7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" t="s">
+        <v>120</v>
+      </c>
+      <c r="G7" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B8" t="s">
+        <v>221</v>
+      </c>
+      <c r="D8" t="s">
+        <v>214</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F8" t="s">
+        <v>120</v>
+      </c>
+      <c r="G8" t="s">
+        <v>215</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="32.28515625" customWidth="1"/>
-    <col min="3" max="3" width="19.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.33203125" customWidth="1"/>
+    <col min="3" max="3" width="19.5546875" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>67</v>
       </c>
@@ -2123,7 +2347,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
         <v>54</v>
       </c>
@@ -2143,7 +2367,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>53</v>
       </c>
@@ -2163,7 +2387,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>183</v>
       </c>
@@ -2180,7 +2404,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>183</v>
       </c>
@@ -2197,7 +2421,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>183</v>
       </c>
@@ -2230,13 +2454,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="55.42578125" customWidth="1"/>
+    <col min="2" max="2" width="55.44140625" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2256,7 +2480,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>20118</v>
       </c>
@@ -2276,7 +2500,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>26410</v>
       </c>
@@ -2296,7 +2520,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>26427</v>
       </c>
@@ -2316,7 +2540,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>26426</v>
       </c>
@@ -2358,13 +2582,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="48.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.140625" customWidth="1"/>
+    <col min="2" max="2" width="48.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2384,7 +2608,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>845</v>
       </c>
@@ -2404,7 +2628,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>6138</v>
       </c>
@@ -2424,7 +2648,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>6142</v>
       </c>
@@ -2444,7 +2668,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>20119</v>
       </c>
@@ -2464,7 +2688,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>3426</v>
       </c>
@@ -2484,7 +2708,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>826</v>
       </c>
@@ -2532,14 +2756,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="35.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2559,7 +2783,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1767</v>
       </c>
@@ -2579,7 +2803,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>20022</v>
       </c>
@@ -2599,7 +2823,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>120</v>
       </c>
@@ -2619,7 +2843,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>1677</v>
       </c>
@@ -2639,7 +2863,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>20115</v>
       </c>
@@ -2659,7 +2883,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>1647</v>
       </c>
@@ -2679,7 +2903,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>1707</v>
       </c>
@@ -2699,7 +2923,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>1787</v>
       </c>
@@ -2753,17 +2977,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="32.28515625" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" customWidth="1"/>
+    <col min="2" max="2" width="32.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.109375" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>67</v>
       </c>
@@ -2783,7 +3007,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>20116</v>
       </c>
@@ -2803,7 +3027,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="11">
         <v>1558</v>
       </c>
@@ -2823,7 +3047,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2178</v>
       </c>
@@ -2843,7 +3067,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
         <v>137</v>
       </c>
@@ -2863,7 +3087,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="13">
         <v>20003</v>
       </c>
@@ -2883,7 +3107,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="11">
         <v>6146</v>
       </c>
@@ -2903,7 +3127,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
         <v>2188</v>
       </c>
@@ -2923,7 +3147,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
         <v>2100</v>
       </c>
@@ -2943,7 +3167,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="13">
         <v>2090</v>
       </c>
@@ -3000,14 +3224,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.140625" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" customWidth="1"/>
+    <col min="4" max="4" width="23.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>67</v>
       </c>
@@ -3027,7 +3251,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="11">
         <v>1050</v>
       </c>
@@ -3047,7 +3271,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="11">
         <v>1060</v>
       </c>
@@ -3067,7 +3291,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -3075,7 +3299,7 @@
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -3083,7 +3307,7 @@
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -3091,7 +3315,7 @@
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -3113,16 +3337,14 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="2" max="2" width="57.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3142,199 +3364,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1160</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" t="s">
-        <v>106</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>1170</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>1180</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" t="s">
-        <v>108</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>1190</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5" t="s">
-        <v>109</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>1200</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>1210</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>1220</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" t="s">
-        <v>112</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>100580</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D9" t="s">
-        <v>140</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1160" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1160" xr:uid="{00000000-0004-0000-0700-000001000000}"/>
-    <hyperlink ref="A3" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1170" xr:uid="{00000000-0004-0000-0700-000002000000}"/>
-    <hyperlink ref="B3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1170" xr:uid="{00000000-0004-0000-0700-000003000000}"/>
-    <hyperlink ref="A4" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1180" xr:uid="{00000000-0004-0000-0700-000004000000}"/>
-    <hyperlink ref="B4" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1180" xr:uid="{00000000-0004-0000-0700-000005000000}"/>
-    <hyperlink ref="A5" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1190" xr:uid="{00000000-0004-0000-0700-000006000000}"/>
-    <hyperlink ref="B5" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1190" xr:uid="{00000000-0004-0000-0700-000007000000}"/>
-    <hyperlink ref="A6" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1200" xr:uid="{00000000-0004-0000-0700-000008000000}"/>
-    <hyperlink ref="B6" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1200" xr:uid="{00000000-0004-0000-0700-000009000000}"/>
-    <hyperlink ref="A7" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1210" xr:uid="{00000000-0004-0000-0700-00000A000000}"/>
-    <hyperlink ref="B7" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1210" xr:uid="{00000000-0004-0000-0700-00000B000000}"/>
-    <hyperlink ref="A8" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1220" xr:uid="{00000000-0004-0000-0700-00000C000000}"/>
-    <hyperlink ref="B8" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1220" xr:uid="{00000000-0004-0000-0700-00000D000000}"/>
-    <hyperlink ref="A9" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=100580" xr:uid="{00000000-0004-0000-0700-00000E000000}"/>
-    <hyperlink ref="B9" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=100580" xr:uid="{00000000-0004-0000-0700-00000F000000}"/>
-    <hyperlink ref="C9" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100100" xr:uid="{00000000-0004-0000-0700-000010000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId18"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="57.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>90012</v>
       </c>
@@ -3354,7 +3384,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>4079</v>
       </c>
@@ -3374,7 +3404,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>102</v>
       </c>
@@ -3394,7 +3424,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4080</v>
       </c>
@@ -3414,7 +3444,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>23099</v>
       </c>
@@ -3434,7 +3464,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>21001</v>
       </c>
@@ -3454,7 +3484,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>46</v>
       </c>
@@ -3474,7 +3504,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>47</v>
       </c>
@@ -3494,7 +3524,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>3063</v>
       </c>
@@ -3514,7 +3544,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>3062</v>
       </c>
@@ -3534,7 +3564,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>3064</v>
       </c>
@@ -3594,7 +3624,209 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.88671875" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>1160</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1170</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1180</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1190</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1200</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" t="s">
+        <v>110</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1210</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1220</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>100580</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1160" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1160" xr:uid="{00000000-0004-0000-0700-000001000000}"/>
+    <hyperlink ref="A3" r:id="rId3" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1170" xr:uid="{00000000-0004-0000-0700-000002000000}"/>
+    <hyperlink ref="B3" r:id="rId4" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1170" xr:uid="{00000000-0004-0000-0700-000003000000}"/>
+    <hyperlink ref="A4" r:id="rId5" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1180" xr:uid="{00000000-0004-0000-0700-000004000000}"/>
+    <hyperlink ref="B4" r:id="rId6" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1180" xr:uid="{00000000-0004-0000-0700-000005000000}"/>
+    <hyperlink ref="A5" r:id="rId7" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1190" xr:uid="{00000000-0004-0000-0700-000006000000}"/>
+    <hyperlink ref="B5" r:id="rId8" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1190" xr:uid="{00000000-0004-0000-0700-000007000000}"/>
+    <hyperlink ref="A6" r:id="rId9" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1200" xr:uid="{00000000-0004-0000-0700-000008000000}"/>
+    <hyperlink ref="B6" r:id="rId10" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1200" xr:uid="{00000000-0004-0000-0700-000009000000}"/>
+    <hyperlink ref="A7" r:id="rId11" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1210" xr:uid="{00000000-0004-0000-0700-00000A000000}"/>
+    <hyperlink ref="B7" r:id="rId12" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1210" xr:uid="{00000000-0004-0000-0700-00000B000000}"/>
+    <hyperlink ref="A8" r:id="rId13" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1220" xr:uid="{00000000-0004-0000-0700-00000C000000}"/>
+    <hyperlink ref="B8" r:id="rId14" display="https://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=1220" xr:uid="{00000000-0004-0000-0700-00000D000000}"/>
+    <hyperlink ref="A9" r:id="rId15" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=100580" xr:uid="{00000000-0004-0000-0700-00000E000000}"/>
+    <hyperlink ref="B9" r:id="rId16" display="https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=100580" xr:uid="{00000000-0004-0000-0700-00000F000000}"/>
+    <hyperlink ref="C9" r:id="rId17" display="https://biobank.ndph.ox.ac.uk/showcase/label.cgi?id=100100" xr:uid="{00000000-0004-0000-0700-000010000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId18"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002D5D40E36B58B0418A5C0DC6F6A2845B" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a816bc34d4292327d4a371c81c74c3a5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xmlns:ns4="301edac2-2a5a-4564-9129-5d780cc3d1d3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="773e6490813a0ac7eb54afe68e0456d4" ns3:_="" ns4:_="">
     <xsd:import namespace="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
@@ -3809,14 +4041,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="bf730ed8-b462-4811-b6bf-a8f46aa7e706" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3827,6 +4051,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD47ECBE-2CA4-4905-9B25-5B5DD8B09919}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3845,23 +4086,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349740AB-8131-4E4B-BDB3-4D33FF056410}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="bf730ed8-b462-4811-b6bf-a8f46aa7e706"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="301edac2-2a5a-4564-9129-5d780cc3d1d3"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6985D056-78E3-4B1E-813E-A88121763A27}">
   <ds:schemaRefs>

</xml_diff>